<commit_message>
Added a new linear regression model
</commit_message>
<xml_diff>
--- a/Sample data for 5mm (34_).xlsx
+++ b/Sample data for 5mm (34_).xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Margi\Desktop\BE PROJECT\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Neevan\Documents\Printing - Research Internship\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F485DAEB-300A-474D-803B-0BC0A12E1E5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14380" windowHeight="3680"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -32,9 +33,6 @@
     <t>Job Number</t>
   </si>
   <si>
-    <t>Paper Type</t>
-  </si>
-  <si>
     <t>Zone number</t>
   </si>
   <si>
@@ -47,9 +45,6 @@
     <t>Delta E before</t>
   </si>
   <si>
-    <t xml:space="preserve">Delta E after </t>
-  </si>
-  <si>
     <t>initial density</t>
   </si>
   <si>
@@ -69,12 +64,18 @@
   </si>
   <si>
     <t>5mm</t>
+  </si>
+  <si>
+    <t>Paper type</t>
+  </si>
+  <si>
+    <t>Delta E after</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -100,12 +101,27 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -114,7 +130,9 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -394,24 +412,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.81640625" customWidth="1"/>
-    <col min="2" max="2" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7265625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.77734375" customWidth="1"/>
+    <col min="2" max="2" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.77734375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="11" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.1796875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="17.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.21875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -419,37 +437,37 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>11</v>
-      </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>4</v>
       </c>
@@ -457,16 +475,16 @@
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="G2">
         <v>5.2</v>

</xml_diff>